<commit_message>
chore: snapshot working tree before residual metrics worktree
</commit_message>
<xml_diff>
--- a/others/Microfluidic_Experiment_Template.xlsb.xlsx
+++ b/others/Microfluidic_Experiment_Template.xlsb.xlsx
@@ -5,24 +5,24 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00 Claude Code\01 MATLAB CODE\01 Microfluid\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00 Claude Code\01 MATLAB CODE\01 Microfluid\others\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{0B68B27C-4BB5-4396-BB00-2AACE9689B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3E66B1D-422B-4D0A-892B-860889818734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="说明 (ReadMe)" sheetId="1" r:id="rId1"/>
     <sheet name="列表与参数 (Lists)" sheetId="2" r:id="rId2"/>
     <sheet name="数据记录 (Data Record)" sheetId="3" r:id="rId3"/>
     <sheet name="分析图表 (Analysis Charts)" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'数据记录 (Data Record)'!$A$1:$P$106</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="132">
   <si>
     <t>微流控 NAPL 驱替实验数据记录模板</t>
   </si>
@@ -66,15 +66,6 @@
     <t>公式说明</t>
   </si>
   <si>
-    <t>F列  Ca = mu_w * v / sigma, 其中 v = Q / (W * D)  -- 芯片参数 W, D 在"列表与参数"表 E8:E9</t>
-  </si>
-  <si>
-    <t>G列  log10(Ca) = LOG10(F列)  -- 毛细数的对数，用于绘制CDC曲线</t>
-  </si>
-  <si>
-    <t>J列  黏度比 M = H列(mu_w) / I列(mu_o)  -- 驱替相与被驱相的黏度比</t>
-  </si>
-  <si>
     <t>参考文献</t>
   </si>
   <si>
@@ -87,21 +78,12 @@
     <t>图表指南</t>
   </si>
   <si>
-    <t>图一：CDC 曲线 -- X: log10(Ca) (G列), Y: S_nr (K列) -&gt; 散点图 + 趋势线</t>
-  </si>
-  <si>
-    <t>图二：Lenormand 相图 -- X: log10(Ca) (G列), Y: M (J列, 对数Y轴) -&gt; 按流型分色散点</t>
-  </si>
-  <si>
     <t>图三：多条件 S_nr 对比 -- 数据透视图, 类别=结构类型, 值=平均S_nr -&gt; 柱状图</t>
   </si>
   <si>
     <t>实验流程闭环</t>
   </si>
   <si>
-    <t>实验台 -&gt; 图像采集 -&gt; MATLAB/Python 脚本提取 S_nr/num_clusters/avg_area -&gt; 填入本表 -&gt; 公式自动算 logCa &amp; M -&gt; 切到图表页刷新 -&gt; 截图汇报</t>
-  </si>
-  <si>
     <t>结构类型</t>
   </si>
   <si>
@@ -136,18 +118,6 @@
   </si>
   <si>
     <t>芯片参数</t>
-  </si>
-  <si>
-    <t>通道宽度 W (um)</t>
-  </si>
-  <si>
-    <t>通道深度 D (um)</t>
-  </si>
-  <si>
-    <t>单位换算系数</t>
-  </si>
-  <si>
-    <t>Ca = mu_w*Q / (sigma*W*D) * k</t>
   </si>
   <si>
     <t>实验编号
@@ -166,14 +136,6 @@
 (uL/min)</t>
   </si>
   <si>
-    <t>毛细数 Ca
-(-) [auto]</t>
-  </si>
-  <si>
-    <t>log10(Ca)
-(-) [auto]</t>
-  </si>
-  <si>
     <t>驱替相黏度 mu_w
 (mPa s)</t>
   </si>
@@ -418,13 +380,132 @@
   </si>
   <si>
     <t>Test3-3</t>
+  </si>
+  <si>
+    <t>F列  名义毛细数 Ca_nom = mu_w * Q / (sigma * W_domain * H) * k，其中 W_domain 和 H 为整体流动域尺度，参数位于"列表与参数"表 E8:E9</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>G列  log10(Ca_nom) = LOG10(F列)  -- 名义毛细数的对数，用于跨工况比较</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>J列  黏度比 M = H列(mu_w) / I列(mu_o)  -- 驱替相与被驱相的黏度比</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>图一：名义 CDC 曲线 -- X: log10(Ca_nom) (G列), Y: S_nr (K列) -&gt; 散点图 + 趋势线</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>图二：名义 Lenormand 相图 -- X: log10(Ca_nom) (G列), Y: M (J列, 对数Y轴) -&gt; 按流型分色散点</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>实验台 -&gt; 图像采集 -&gt; MATLAB/Python 脚本提取 S_nr/num_clusters/avg_area -&gt; 填入本表 -&gt; 公式自动算 log10(Ca_nom) &amp; M -&gt; 切到图表页刷新 -&gt; 截图汇报</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>流动域宽度 W_domain (um)</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>流动域高度 H (um)</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>单位换算系数 k</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ca_nom = mu_w*Q / (sigma*W_domain*H) * k</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>名义毛细数 Ca_nom
+(-) [auto]</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>log10(Ca_nom)
+(-) [auto]</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dodecane</t>
+  </si>
+  <si>
+    <t>BD</t>
+  </si>
+  <si>
+    <t>BO</t>
+  </si>
+  <si>
+    <t>Q (µL/min)</t>
+  </si>
+  <si>
+    <t>S⁰ₙ</t>
+  </si>
+  <si>
+    <t>ΔSₙ (%)</t>
+  </si>
+  <si>
+    <t>Blobs₀</t>
+  </si>
+  <si>
+    <t>Blobsᵣₑₛ</t>
+  </si>
+  <si>
+    <t>IFL₀ (px)</t>
+  </si>
+  <si>
+    <t>IFLᵣₑₛ (px)</t>
+  </si>
+  <si>
+    <t>t_trans (s)</t>
+  </si>
+  <si>
+    <t>S_residual/S_initoa=V_resisual/V_initial</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>Contaminant</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>ⁿ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ʳᵉˢ</t>
+    </r>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dodecane</t>
+    <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,6 +575,37 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -539,7 +651,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -562,11 +674,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD6D6D6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD6D6D6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFD6D6D6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD6D6D6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -605,9 +735,25 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -688,31 +834,31 @@
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-4.385606274</c:v>
+                  <c:v>-5.156458285</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3.987666265</c:v>
+                  <c:v>-4.85542829</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-3.686636269</c:v>
+                  <c:v>-4.679337031</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.500785173</c:v>
+                  <c:v>-5.271637185</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-4.199755177</c:v>
+                  <c:v>-4.970607189</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-3.801815169</c:v>
+                  <c:v>-4.79451593</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-3.686636269</c:v>
+                  <c:v>-5.131066625</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-3.686636269</c:v>
+                  <c:v>-4.830036629</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-4.059184618</c:v>
+                  <c:v>-4.65394537</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -723,33 +869,6 @@
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="105"/>
-                <c:pt idx="0">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.3821</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.35</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.08</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -936,31 +1055,31 @@
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>-4.385606274</c:v>
+                  <c:v>-5.156458285</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3.987666265</c:v>
+                  <c:v>-4.85542829</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-3.686636269</c:v>
+                  <c:v>-4.679337031</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.500785173</c:v>
+                  <c:v>-5.271637185</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-4.199755177</c:v>
+                  <c:v>-4.970607189</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-3.801815169</c:v>
+                  <c:v>-4.79451593</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-3.686636269</c:v>
+                  <c:v>-5.131066625</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-3.686636269</c:v>
+                  <c:v>-4.830036629</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-4.059184618</c:v>
+                  <c:v>-4.65394537</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -990,13 +1109,13 @@
                   <c:v>0.74626865671641784</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.47619047619047616</c:v>
+                  <c:v>0.7142857142857143</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.47619047619047616</c:v>
+                  <c:v>0.7142857142857143</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.47619047619047616</c:v>
+                  <c:v>0.7142857142857143</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1501,33 +1620,6 @@
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.3821</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.35</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.08</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1640,6 +1732,1176 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Dodecane</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$2:$F$4</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.35381355932203395</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.32950990615224196</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.30489073881373568</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-F6F1-4034-AAB3-80A7541ADAEC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>1-BD</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$5:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$5:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.3950892857142857</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.36723768736616702</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.27772020725388602</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-F6F1-4034-AAB3-80A7541ADAEC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>1-BO</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$8:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$8:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.31578947368421051</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.24374319912948858</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.16934619506966772</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-F6F1-4034-AAB3-80A7541ADAEC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="922969519"/>
+        <c:axId val="922969999"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="922969519"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="6"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US"/>
+                  <a:t>流速</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB" altLang="zh-CN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="922969999"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="1"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="922969999"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US"/>
+                  <a:t>残余</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:t>NAPL</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB" altLang="zh-CN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="922969519"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$5:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$I$5:$I$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>244</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>265</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1D55-4CCF-B592-7EEB339B56D6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$I$2:$I$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>319</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>338</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>387</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-1D55-4CCF-B592-7EEB339B56D6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$8:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$I$8:$I$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>241</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>245</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>302</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-1D55-4CCF-B592-7EEB339B56D6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="922969519"/>
+        <c:axId val="922969999"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="922969519"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="922969999"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="922969999"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="922969519"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$5:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$K$5:$K$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>257.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>263.7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>281.39999999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-92F1-4468-96FF-02B8F7DCE638}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$K$2:$K$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>260.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>307.39999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>279.10000000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-92F1-4468-96FF-02B8F7DCE638}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$C$8:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$K$8:$K$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>188.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>181.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-92F1-4468-96FF-02B8F7DCE638}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="922969519"/>
+        <c:axId val="922969999"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="922969519"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="922969999"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="922969999"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="922969519"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1737,6 +2999,123 @@
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>390767</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>107463</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>68382</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>21493</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B87E767-55D3-6A3C-7CE6-9E994E2BC9D8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>691660</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>96228</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>938822</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>155820</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1127B9FC-5713-4A4F-96D8-1C0C3E19E33E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>414704</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>103066</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>385397</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>30285</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4605DEE3-6C59-4C75-8CF3-7E9A01843F6B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -2088,62 +3467,62 @@
     </row>
     <row r="11" spans="1:1" ht="26" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>8</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>9</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="26" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="26" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="26" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>16</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="26" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2166,27 +3545,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="E2" s="5">
         <v>72</v>
@@ -2194,13 +3573,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="E3" s="5">
         <v>52.8</v>
@@ -2208,13 +3587,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E4" s="5">
         <v>40.5</v>
@@ -2222,10 +3601,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E5" s="5">
         <v>38.200000000000003</v>
@@ -2233,7 +3612,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -2241,20 +3620,20 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D7" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" s="6" t="s">
-        <v>32</v>
+        <v>111</v>
       </c>
       <c r="E8" s="7">
-        <v>500</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D9" s="6" t="s">
-        <v>33</v>
+        <v>112</v>
       </c>
       <c r="E9" s="7">
         <v>20</v>
@@ -2262,7 +3641,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D10" s="6" t="s">
-        <v>34</v>
+        <v>113</v>
       </c>
       <c r="E10" s="7">
         <f>1000/60</f>
@@ -2271,12 +3650,12 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D11" s="8" t="s">
-        <v>35</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
@@ -2285,39 +3664,39 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="E15" s="15"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="B16" s="15">
         <v>170.34</v>
@@ -2329,27 +3708,27 @@
         <v>193.13</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E17" s="15"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B18" s="15">
         <v>0.749</v>
@@ -2361,12 +3740,12 @@
         <v>1.117</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="B19" s="15">
         <v>1.34</v>
@@ -2375,15 +3754,15 @@
         <v>3.7</v>
       </c>
       <c r="D19" s="15">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="B20" s="15">
         <v>52.8</v>
@@ -2395,29 +3774,29 @@
         <v>38.200000000000003</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="D21" s="15">
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="B22" s="16">
         <v>4.8E-10</v>
@@ -2429,29 +3808,29 @@
         <v>5.1999999999999996E-10</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="B24" s="15">
         <v>3.4000000000000002E-2</v>
@@ -2463,12 +3842,12 @@
         <v>0.13300000000000001</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B25" s="15">
         <v>25.35</v>
@@ -2480,12 +3859,12 @@
         <v>27.8</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="B26" s="15">
         <v>71</v>
@@ -2497,12 +3876,12 @@
         <v>62</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B27" s="15">
         <v>1.421</v>
@@ -2517,46 +3896,46 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="E28" s="15"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="E29" s="15"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E30" s="15"/>
     </row>
@@ -2569,7 +3948,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -2605,77 +3984,75 @@
   <sheetData>
     <row r="1" spans="1:16" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="9" t="s">
+      <c r="O1" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="P1" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N1" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C2" s="10"/>
       <c r="D2" s="5">
         <v>40.5</v>
       </c>
       <c r="E2" s="17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" s="11">
         <f>IFERROR((H2*E2) / (D2*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>4.11522633744856E-5</v>
+        <v>6.9749598939806103E-6</v>
       </c>
       <c r="G2" s="12">
         <f t="shared" ref="G2:G39" si="0">IFERROR(LOG10(F2),"")</f>
-        <v>-4.3856062735983121</v>
+        <v>-5.1564582852404559</v>
       </c>
       <c r="H2" s="10">
         <v>1</v>
@@ -2687,48 +4064,38 @@
         <f t="shared" ref="J2:J39" si="1">IFERROR(H2/I2,"")</f>
         <v>0.27027027027027023</v>
       </c>
-      <c r="K2" s="13">
-        <v>0.12</v>
-      </c>
-      <c r="L2" s="10">
-        <v>0.45</v>
-      </c>
-      <c r="M2" s="10">
-        <v>15</v>
-      </c>
-      <c r="N2" s="10">
-        <v>3000</v>
-      </c>
+      <c r="K2" s="13"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
       <c r="O2" s="10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C3" s="10"/>
       <c r="D3" s="5">
         <v>40.5</v>
       </c>
       <c r="E3" s="17">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="F3" s="11">
         <f>IFERROR((H3*E3) / (D3*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>1.0288065843621399E-4</v>
+        <v>1.3949919787961221E-5</v>
       </c>
       <c r="G3" s="12">
         <f t="shared" ref="G3:G8" si="2">IFERROR(LOG10(F3),"")</f>
-        <v>-3.9876662649262746</v>
+        <v>-4.8554282895764755</v>
       </c>
       <c r="H3" s="10">
         <v>1</v>
@@ -2740,48 +4107,38 @@
         <f t="shared" ref="J3:J8" si="3">IFERROR(H3/I3,"")</f>
         <v>0.27027027027027023</v>
       </c>
-      <c r="K3" s="13">
-        <v>0.12</v>
-      </c>
-      <c r="L3" s="10">
-        <v>0.85</v>
-      </c>
-      <c r="M3" s="10">
-        <v>3</v>
-      </c>
-      <c r="N3" s="10">
-        <v>500</v>
-      </c>
+      <c r="K3" s="13"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
       <c r="O3" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P3" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C4" s="10"/>
       <c r="D4" s="5">
         <v>40.5</v>
       </c>
       <c r="E4" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F4" s="11">
         <f>IFERROR((H4*E4) / (D4*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>2.0576131687242798E-4</v>
+        <v>2.0924879681941831E-5</v>
       </c>
       <c r="G4" s="12">
         <f t="shared" si="2"/>
-        <v>-3.6866362692622934</v>
+        <v>-4.6793370305207942</v>
       </c>
       <c r="H4" s="10">
         <v>1</v>
@@ -2793,48 +4150,38 @@
         <f t="shared" si="3"/>
         <v>0.27027027027027023</v>
       </c>
-      <c r="K4" s="13">
-        <v>0.3821</v>
-      </c>
-      <c r="L4" s="10">
-        <v>0.85</v>
-      </c>
-      <c r="M4" s="10">
-        <v>3</v>
-      </c>
-      <c r="N4" s="10">
-        <v>500</v>
-      </c>
+      <c r="K4" s="13"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
       <c r="O4" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C5" s="10"/>
       <c r="D5" s="5">
         <v>52.8</v>
       </c>
       <c r="E5" s="17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR((H5*E5) / (D5*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>3.1565656565656566E-5</v>
+        <v>5.3501112823146726E-6</v>
       </c>
       <c r="G5" s="12">
         <f t="shared" si="2"/>
-        <v>-4.5007851729174559</v>
+        <v>-5.2716371845595997</v>
       </c>
       <c r="H5" s="10">
         <v>1</v>
@@ -2846,48 +4193,38 @@
         <f t="shared" si="3"/>
         <v>0.74626865671641784</v>
       </c>
-      <c r="K5" s="13">
-        <v>0.35</v>
-      </c>
-      <c r="L5" s="10">
-        <v>0.45</v>
-      </c>
-      <c r="M5" s="10">
-        <v>15</v>
-      </c>
-      <c r="N5" s="10">
-        <v>3000</v>
-      </c>
+      <c r="K5" s="13"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
       <c r="O5" s="10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C6" s="10"/>
       <c r="D6" s="5">
         <v>52.8</v>
       </c>
       <c r="E6" s="17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6" s="11">
         <f>IFERROR((H6*E6) / (D6*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>6.3131313131313131E-5</v>
+        <v>1.0700222564629345E-5</v>
       </c>
       <c r="G6" s="12">
         <f t="shared" si="2"/>
-        <v>-4.1997551772534747</v>
+        <v>-4.9706071888956185</v>
       </c>
       <c r="H6" s="10">
         <v>1</v>
@@ -2899,48 +4236,38 @@
         <f t="shared" si="3"/>
         <v>0.74626865671641784</v>
       </c>
-      <c r="K6" s="13">
-        <v>0.12</v>
-      </c>
-      <c r="L6" s="10">
-        <v>0.85</v>
-      </c>
-      <c r="M6" s="10">
-        <v>3</v>
-      </c>
-      <c r="N6" s="10">
-        <v>500</v>
-      </c>
+      <c r="K6" s="13"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
       <c r="O6" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C7" s="10"/>
       <c r="D7" s="5">
         <v>52.8</v>
       </c>
       <c r="E7" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" s="11">
         <f>IFERROR((H7*E7) / (D7*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>1.5782828282828284E-4</v>
+        <v>1.6050333846944017E-5</v>
       </c>
       <c r="G7" s="12">
         <f t="shared" si="2"/>
-        <v>-3.8018151685814372</v>
+        <v>-4.794515929839938</v>
       </c>
       <c r="H7" s="10">
         <v>1</v>
@@ -2952,182 +4279,144 @@
         <f t="shared" si="3"/>
         <v>0.74626865671641784</v>
       </c>
-      <c r="K7" s="13">
-        <v>0.12</v>
-      </c>
-      <c r="L7" s="10">
-        <v>0.85</v>
-      </c>
-      <c r="M7" s="10">
-        <v>3</v>
-      </c>
-      <c r="N7" s="10">
-        <v>500</v>
-      </c>
+      <c r="K7" s="13"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
       <c r="O7" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="10">
-        <v>30</v>
-      </c>
-      <c r="D8" s="5">
-        <v>40.5</v>
-      </c>
-      <c r="E8" s="10">
-        <v>5</v>
+        <v>39</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10">
+        <v>38.200000000000003</v>
+      </c>
+      <c r="E8" s="17">
+        <v>2</v>
       </c>
       <c r="F8" s="11">
         <f>IFERROR((H8*E8) / (D8*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>2.0576131687242798E-4</v>
+        <v>7.3949182122045717E-6</v>
       </c>
       <c r="G8" s="12">
         <f t="shared" si="2"/>
-        <v>-3.6866362692622934</v>
+        <v>-5.131066624937497</v>
       </c>
       <c r="H8" s="10">
         <v>1</v>
       </c>
       <c r="I8" s="10">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="J8" s="12">
         <f t="shared" si="3"/>
-        <v>0.47619047619047616</v>
-      </c>
-      <c r="K8" s="13">
-        <v>0.12</v>
-      </c>
-      <c r="L8" s="10">
-        <v>0.85</v>
-      </c>
-      <c r="M8" s="10">
-        <v>3</v>
-      </c>
-      <c r="N8" s="10">
-        <v>500</v>
-      </c>
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="K8" s="13"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
       <c r="O8" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C9" s="10"/>
       <c r="D9" s="10">
-        <v>40.5</v>
-      </c>
-      <c r="E9" s="10">
-        <v>5</v>
+        <v>38.200000000000003</v>
+      </c>
+      <c r="E9" s="17">
+        <v>4</v>
       </c>
       <c r="F9" s="11">
         <f>IFERROR((H9*E9) / (D9*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>2.0576131687242798E-4</v>
+        <v>1.4789836424409143E-5</v>
       </c>
       <c r="G9" s="12">
         <f t="shared" si="0"/>
-        <v>-3.6866362692622934</v>
+        <v>-4.8300366292735157</v>
       </c>
       <c r="H9" s="10">
         <v>1</v>
       </c>
       <c r="I9" s="10">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="J9" s="12">
         <f t="shared" si="1"/>
-        <v>0.47619047619047616</v>
-      </c>
-      <c r="K9" s="13">
-        <v>0.12</v>
-      </c>
-      <c r="L9" s="10">
-        <v>0.85</v>
-      </c>
-      <c r="M9" s="10">
-        <v>3</v>
-      </c>
-      <c r="N9" s="10">
-        <v>500</v>
-      </c>
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="K9" s="13"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
       <c r="O9" s="10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="10">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C10" s="10"/>
       <c r="D10" s="10">
         <v>38.200000000000003</v>
       </c>
       <c r="E10" s="10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F10" s="11">
         <f>IFERROR((H10*E10) / (D10*'列表与参数 (Lists)'!$E$8*'列表与参数 (Lists)'!$E$9) * '列表与参数 (Lists)'!$E$10,"")</f>
-        <v>8.7260034904013966E-5</v>
+        <v>2.2184754636613716E-5</v>
       </c>
       <c r="G10" s="12">
         <f t="shared" si="0"/>
-        <v>-4.0591846176313711</v>
+        <v>-4.6539453702178344</v>
       </c>
       <c r="H10" s="10">
         <v>1</v>
       </c>
       <c r="I10" s="10">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="J10" s="12">
         <f t="shared" si="1"/>
-        <v>0.47619047619047616</v>
-      </c>
-      <c r="K10" s="13">
-        <v>0.08</v>
-      </c>
-      <c r="L10" s="10">
-        <v>0.92</v>
-      </c>
-      <c r="M10" s="10">
-        <v>2</v>
-      </c>
-      <c r="N10" s="10">
-        <v>250</v>
-      </c>
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="K10" s="13"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
       <c r="O10" s="10" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -4523,8 +5812,671 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>50</v>
-      </c>
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C455A02D-81BC-45D7-A1B3-E4C3676516AE}">
+  <dimension ref="B1:L20"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="8.7265625" style="18"/>
+    <col min="5" max="5" width="9.54296875" style="18" customWidth="1"/>
+    <col min="6" max="6" width="54.26953125" style="18" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="18" customWidth="1"/>
+    <col min="8" max="8" width="12.08984375" style="18" customWidth="1"/>
+    <col min="9" max="9" width="13" style="18" customWidth="1"/>
+    <col min="10" max="10" width="15.81640625" style="18" customWidth="1"/>
+    <col min="11" max="11" width="18.54296875" style="18" customWidth="1"/>
+    <col min="12" max="12" width="17.6328125" style="18" customWidth="1"/>
+    <col min="13" max="16384" width="8.7265625" style="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="J1" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="L1" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="22">
+        <v>2</v>
+      </c>
+      <c r="D2" s="18">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="E2" s="18">
+        <v>0.33400000000000002</v>
+      </c>
+      <c r="F2" s="19">
+        <f>E2/D2</f>
+        <v>0.35381355932203395</v>
+      </c>
+      <c r="G2" s="19">
+        <f>D2-E2</f>
+        <v>0.60999999999999988</v>
+      </c>
+      <c r="H2" s="18">
+        <v>15</v>
+      </c>
+      <c r="I2" s="18">
+        <v>319</v>
+      </c>
+      <c r="J2" s="18">
+        <v>59.2</v>
+      </c>
+      <c r="K2" s="18">
+        <v>260.5</v>
+      </c>
+      <c r="L2" s="18">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="22">
+        <v>4</v>
+      </c>
+      <c r="D3" s="18">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="E3" s="18">
+        <v>0.316</v>
+      </c>
+      <c r="F3" s="19">
+        <f t="shared" ref="F3:F10" si="0">E3/D3</f>
+        <v>0.32950990615224196</v>
+      </c>
+      <c r="G3" s="19">
+        <f t="shared" ref="G3:G10" si="1">D3-E3</f>
+        <v>0.64300000000000002</v>
+      </c>
+      <c r="H3" s="18">
+        <v>9</v>
+      </c>
+      <c r="I3" s="18">
+        <v>338</v>
+      </c>
+      <c r="J3" s="18">
+        <v>56.1</v>
+      </c>
+      <c r="K3" s="18">
+        <v>307.39999999999998</v>
+      </c>
+      <c r="L3" s="18">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="22">
+        <v>6</v>
+      </c>
+      <c r="D4" s="18">
+        <v>0.96099999999999997</v>
+      </c>
+      <c r="E4" s="18">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="F4" s="19">
+        <f t="shared" si="0"/>
+        <v>0.30489073881373568</v>
+      </c>
+      <c r="G4" s="19">
+        <f t="shared" si="1"/>
+        <v>0.66799999999999993</v>
+      </c>
+      <c r="H4" s="18">
+        <v>11</v>
+      </c>
+      <c r="I4" s="18">
+        <v>387</v>
+      </c>
+      <c r="J4" s="18">
+        <v>41.3</v>
+      </c>
+      <c r="K4" s="18">
+        <v>279.10000000000002</v>
+      </c>
+      <c r="L4" s="18">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="22">
+        <v>2</v>
+      </c>
+      <c r="D5" s="18">
+        <v>0.89600000000000002</v>
+      </c>
+      <c r="E5" s="18">
+        <v>0.35399999999999998</v>
+      </c>
+      <c r="F5" s="19">
+        <f t="shared" si="0"/>
+        <v>0.3950892857142857</v>
+      </c>
+      <c r="G5" s="19">
+        <f t="shared" si="1"/>
+        <v>0.54200000000000004</v>
+      </c>
+      <c r="H5" s="18">
+        <v>22</v>
+      </c>
+      <c r="I5" s="18">
+        <v>198</v>
+      </c>
+      <c r="J5" s="18">
+        <v>98.9</v>
+      </c>
+      <c r="K5" s="18">
+        <v>257.2</v>
+      </c>
+      <c r="L5" s="18">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="22">
+        <v>4</v>
+      </c>
+      <c r="D6" s="18">
+        <v>0.93400000000000005</v>
+      </c>
+      <c r="E6" s="18">
+        <v>0.34300000000000003</v>
+      </c>
+      <c r="F6" s="19">
+        <f t="shared" si="0"/>
+        <v>0.36723768736616702</v>
+      </c>
+      <c r="G6" s="19">
+        <f t="shared" si="1"/>
+        <v>0.59099999999999997</v>
+      </c>
+      <c r="H6" s="18">
+        <v>16</v>
+      </c>
+      <c r="I6" s="18">
+        <v>244</v>
+      </c>
+      <c r="J6" s="18">
+        <v>79.3</v>
+      </c>
+      <c r="K6" s="18">
+        <v>263.7</v>
+      </c>
+      <c r="L6" s="18">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="22">
+        <v>6</v>
+      </c>
+      <c r="D7" s="18">
+        <v>0.96499999999999997</v>
+      </c>
+      <c r="E7" s="18">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="F7" s="19">
+        <f t="shared" si="0"/>
+        <v>0.27772020725388602</v>
+      </c>
+      <c r="G7" s="19">
+        <f t="shared" si="1"/>
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="H7" s="18">
+        <v>11</v>
+      </c>
+      <c r="I7" s="18">
+        <v>265</v>
+      </c>
+      <c r="J7" s="18">
+        <v>50.5</v>
+      </c>
+      <c r="K7" s="18">
+        <v>281.39999999999998</v>
+      </c>
+      <c r="L7" s="18">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="22">
+        <v>2</v>
+      </c>
+      <c r="D8" s="18">
+        <v>0.95</v>
+      </c>
+      <c r="E8" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="F8" s="19">
+        <f t="shared" si="0"/>
+        <v>0.31578947368421051</v>
+      </c>
+      <c r="G8" s="19">
+        <f t="shared" si="1"/>
+        <v>0.64999999999999991</v>
+      </c>
+      <c r="H8" s="18">
+        <v>15</v>
+      </c>
+      <c r="I8" s="18">
+        <v>241</v>
+      </c>
+      <c r="J8" s="18">
+        <v>52.2</v>
+      </c>
+      <c r="K8" s="18">
+        <v>188.4</v>
+      </c>
+      <c r="L8" s="18">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="22">
+        <v>4</v>
+      </c>
+      <c r="D9" s="18">
+        <v>0.91900000000000004</v>
+      </c>
+      <c r="E9" s="18">
+        <v>0.224</v>
+      </c>
+      <c r="F9" s="19">
+        <f t="shared" si="0"/>
+        <v>0.24374319912948858</v>
+      </c>
+      <c r="G9" s="19">
+        <f t="shared" si="1"/>
+        <v>0.69500000000000006</v>
+      </c>
+      <c r="H9" s="18">
+        <v>15</v>
+      </c>
+      <c r="I9" s="18">
+        <v>245</v>
+      </c>
+      <c r="J9" s="18">
+        <v>62.5</v>
+      </c>
+      <c r="K9" s="18">
+        <v>195</v>
+      </c>
+      <c r="L9" s="18">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="22">
+        <v>6</v>
+      </c>
+      <c r="D10" s="18">
+        <v>0.93300000000000005</v>
+      </c>
+      <c r="E10" s="18">
+        <v>0.158</v>
+      </c>
+      <c r="F10" s="19">
+        <f t="shared" si="0"/>
+        <v>0.16934619506966772</v>
+      </c>
+      <c r="G10" s="19">
+        <f t="shared" si="1"/>
+        <v>0.77500000000000002</v>
+      </c>
+      <c r="H10" s="18">
+        <v>11</v>
+      </c>
+      <c r="I10" s="18">
+        <v>302</v>
+      </c>
+      <c r="J10" s="18">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="K10" s="18">
+        <v>181.5</v>
+      </c>
+      <c r="L10" s="18">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="22">
+        <v>2</v>
+      </c>
+      <c r="D12" s="22">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="E12" s="22">
+        <v>0.33400000000000002</v>
+      </c>
+      <c r="F12" s="22">
+        <v>0.35</v>
+      </c>
+      <c r="G12" s="22">
+        <v>15</v>
+      </c>
+      <c r="H12" s="22">
+        <v>319</v>
+      </c>
+      <c r="I12" s="22">
+        <v>59.2</v>
+      </c>
+      <c r="J12" s="22">
+        <v>260.5</v>
+      </c>
+      <c r="K12" s="22"/>
+    </row>
+    <row r="13" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="22">
+        <v>4</v>
+      </c>
+      <c r="D13" s="22">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="E13" s="22">
+        <v>0.316</v>
+      </c>
+      <c r="F13" s="22">
+        <v>0.33</v>
+      </c>
+      <c r="G13" s="22">
+        <v>9</v>
+      </c>
+      <c r="H13" s="22">
+        <v>338</v>
+      </c>
+      <c r="I13" s="22">
+        <v>56.1</v>
+      </c>
+      <c r="J13" s="22">
+        <v>307.39999999999998</v>
+      </c>
+      <c r="K13" s="22"/>
+    </row>
+    <row r="14" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" s="22">
+        <v>6</v>
+      </c>
+      <c r="D14" s="22">
+        <v>0.96099999999999997</v>
+      </c>
+      <c r="E14" s="22">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="F14" s="22">
+        <v>0.3</v>
+      </c>
+      <c r="G14" s="22">
+        <v>11</v>
+      </c>
+      <c r="H14" s="22">
+        <v>387</v>
+      </c>
+      <c r="I14" s="22">
+        <v>41.3</v>
+      </c>
+      <c r="J14" s="22">
+        <v>279.10000000000002</v>
+      </c>
+      <c r="K14" s="22"/>
+    </row>
+    <row r="15" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="22">
+        <v>2</v>
+      </c>
+      <c r="D15" s="22">
+        <v>0.89600000000000002</v>
+      </c>
+      <c r="E15" s="22">
+        <v>0.35399999999999998</v>
+      </c>
+      <c r="F15" s="22">
+        <v>0.4</v>
+      </c>
+      <c r="G15" s="22">
+        <v>22</v>
+      </c>
+      <c r="H15" s="22">
+        <v>198</v>
+      </c>
+      <c r="I15" s="22">
+        <v>98.9</v>
+      </c>
+      <c r="J15" s="22">
+        <v>257.2</v>
+      </c>
+      <c r="K15" s="22"/>
+    </row>
+    <row r="16" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="22">
+        <v>4</v>
+      </c>
+      <c r="D16" s="22">
+        <v>0.93400000000000005</v>
+      </c>
+      <c r="E16" s="22">
+        <v>0.34300000000000003</v>
+      </c>
+      <c r="F16" s="22">
+        <v>0.37</v>
+      </c>
+      <c r="G16" s="22">
+        <v>16</v>
+      </c>
+      <c r="H16" s="22">
+        <v>244</v>
+      </c>
+      <c r="I16" s="22">
+        <v>79.3</v>
+      </c>
+      <c r="J16" s="22">
+        <v>263.7</v>
+      </c>
+      <c r="K16" s="22"/>
+    </row>
+    <row r="17" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="22">
+        <v>6</v>
+      </c>
+      <c r="D17" s="22">
+        <v>0.96499999999999997</v>
+      </c>
+      <c r="E17" s="22">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="F17" s="22">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="G17" s="22">
+        <v>11</v>
+      </c>
+      <c r="H17" s="22">
+        <v>265</v>
+      </c>
+      <c r="I17" s="22">
+        <v>50.5</v>
+      </c>
+      <c r="J17" s="22">
+        <v>281.39999999999998</v>
+      </c>
+      <c r="K17" s="22"/>
+    </row>
+    <row r="18" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="22">
+        <v>2</v>
+      </c>
+      <c r="D18" s="22">
+        <v>0.95</v>
+      </c>
+      <c r="E18" s="22">
+        <v>0.3</v>
+      </c>
+      <c r="F18" s="22">
+        <v>0.32</v>
+      </c>
+      <c r="G18" s="22">
+        <v>15</v>
+      </c>
+      <c r="H18" s="22">
+        <v>241</v>
+      </c>
+      <c r="I18" s="22">
+        <v>52.2</v>
+      </c>
+      <c r="J18" s="22">
+        <v>188.4</v>
+      </c>
+      <c r="K18" s="22"/>
+    </row>
+    <row r="19" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="22">
+        <v>4</v>
+      </c>
+      <c r="D19" s="22">
+        <v>0.91900000000000004</v>
+      </c>
+      <c r="E19" s="22">
+        <v>0.224</v>
+      </c>
+      <c r="F19" s="22">
+        <v>0.24</v>
+      </c>
+      <c r="G19" s="22">
+        <v>15</v>
+      </c>
+      <c r="H19" s="22">
+        <v>245</v>
+      </c>
+      <c r="I19" s="22">
+        <v>62.5</v>
+      </c>
+      <c r="J19" s="22">
+        <v>195</v>
+      </c>
+      <c r="K19" s="22"/>
+    </row>
+    <row r="20" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="22">
+        <v>6</v>
+      </c>
+      <c r="D20" s="22">
+        <v>0.93300000000000005</v>
+      </c>
+      <c r="E20" s="22">
+        <v>0.158</v>
+      </c>
+      <c r="F20" s="22">
+        <v>0.17</v>
+      </c>
+      <c r="G20" s="22">
+        <v>11</v>
+      </c>
+      <c r="H20" s="22">
+        <v>302</v>
+      </c>
+      <c r="I20" s="22">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="J20" s="22">
+        <v>181.5</v>
+      </c>
+      <c r="K20" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>

</xml_diff>